<commit_message>
Mark V-TOP tariff classification as confirmed by the client
The client confirmed the 8 Sep 2026 classification table in full, so the
conditional proposals ("Pokud popis odpovida charakteru zbozi...") for
SRCS101/SRCS101D, SR1405 and SR8111 are now closed. Those rows are
flagged as confirmed rather than pending verification, and the open
points list is updated accordingly.

Orange is now reserved for the single CBAM item (7326 90 98 90); the
changed and resolved codes are green. Codes, weights and values are
unchanged: 80,006 pcs, NW 665.95 kg, GW 745.00 kg, EUR 6,069.20.

Still open and noted: the TARIC duty rate for 8528 59 00 90, the missing
preferential origin statement, and that this is a classification proposal
confirmed by the client rather than a binding BTI.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHPYjNmJKeJf7vhfGTd7Gq
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_V_TOP_EUROPE_WPXA26B0812CZ323.xlsx
+++ b/output/HS_Code_Summary_V_TOP_EUROPE_WPXA26B0812CZ323.xlsx
@@ -60,12 +60,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
+        <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
+        <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
     <fill>
@@ -154,8 +154,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -708,183 +708,183 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>ZMĚNA + OVĚŘIT</t>
+          <t>ZMĚNA – POTVRZENO</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>ZMĚNA sazebního zařazení 8. 9. 2026: SRCS101/SRCS101D z 8531 20 00 00 a SR1405 z 8531 20 95 90 → obojí 8528 59 00 90. Obě položky proto nyní tvoří jeden řádek. Návrh je podmíněný: „Pokud popis odpovídá charakteru zboží, pak popisu odpovídá navržený TC kód.“ → nechat potvrdit klientem, že popis (bez HDMI/DP/VGA/DVI vstupu) odpovídá skutečnosti. POZOR: přeřazení z položky 8531 do 8528 59 (monitory) může znamenat výrazně vyšší celní sazbu – ověřit v TARIC k datu podání.</t>
+          <t>ZMĚNA sazebního zařazení 8. 9. 2026: SRCS101/SRCS101D z 8531 20 00 00 a SR1405 z 8531 20 95 90 → obojí 8528 59 00 90. Obě položky proto nyní tvoří jeden řádek. POTVRZENO KLIENTEM 9. 9. 2026 – podmínka návrhu („Pokud popis odpovídá charakteru zboží…“) je splněna, displeje nemají externí obrazový vstup HDMI/DP/VGA/DVI. POZOR: přeřazení z položky 8531 do 8528 59 (monitory) může znamenat výrazně vyšší celní sazbu – ověřit v TARIC k datu podání.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, CN</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>7326 90 98 90</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Stolní kovový nosný stojan ve tvaru T pro uchycení napájecí lišty SR8100 a LCD video tagů, s integrovaným přívodním elektrickým kabelem. Materiál stojanu: železo.</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>SR8170</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="12" t="n">
         <v>1.68</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="12" t="n">
         <v>1.853</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="12" t="n">
         <v>1.932</v>
       </c>
-      <c r="J4" s="9" t="n">
+      <c r="J4" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>CFR Praha</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>CBAM zboží (železo/ocel, příloha I) – JEDINÁ CBAM položka v zásilce, čistá hmotnost 1,68 kg. Příjemce V-TOP EUROPE s.r.o. (EORI CZ25795040) = Y137, do 50 t ročně. Kód doplněn ze 6místného 7326 90 na 7326 90 98 90. Antidumping: u této položky z ČLR není známé opatření – ověřit v TARIC.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, CN</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>8504 40 83 90</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Externí napájecí adaptér pro video tag; převod síťového střídavého napětí na stabilizovaný stejnosměrný výstup 24 V; max. výstupní výkon 24 × 2,5 = 60 W.</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>SR8111</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="8" t="n">
         <v>0.34</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="8" t="n">
         <v>0.375</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="8" t="n">
         <v>0.391</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>CFR Praha</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
-          <t>VYŘEŠENO</t>
-        </is>
-      </c>
-      <c r="M5" s="10" t="inlineStr">
-        <is>
-          <t>Chybějící HS kód DOPLNĚN sazebním zařazením 8. 9. 2026 (dříve „?“). Návrh je podmíněný: „Pokud popis odpovídá charakteru zboží, pak popisu odpovídá navržený TC kód.“ → nechat potvrdit parametry adaptéru (výstup 24 V DC, 60 W).</t>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>VYŘEŠENO – POTVRZENO</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Chybějící HS kód DOPLNĚN sazebním zařazením 8. 9. 2026 (dříve „?“). POTVRZENO KLIENTEM 9. 9. 2026 – podmínka návrhu je splněna, parametry adaptéru (výstup 24 V DC, max. 60 W) odpovídají popisu.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>HANGZHOU ONTIME I.T. CO., LTD., Hangzhou, CN</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>8536 90 01 00</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Horizontální napájecí lišta s měděnými kontakty pro mechanické uchycení a napájení LCD video tagů, 0,5 m. Materiál: hliník, železo a měď.</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>SR8100</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="8" t="n">
         <v>0.28</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="8" t="n">
         <v>0.309</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="8" t="n">
         <v>0.322</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="9" t="n">
         <v>2.2</v>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>CFR Praha</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ZMĚNA – CBAM ODPADÁ</t>
         </is>
       </c>
-      <c r="M6" s="10" t="inlineStr">
-        <is>
-          <t>ZMĚNA sazebního zařazení 8. 9. 2026: z 7616 99 (hliník) → 8536 90 01 00. Zákazník opravil popis: název „magnetic power rail“ byl chybný, nejde o magnetickou hliníkovou lištu, ale o vrchní lištu stojanu s měděnými kontakty (uchycení čistě mechanické). DŮSLEDEK: položka již NENÍ CBAM zboží a odpadá i podezření na antidumping dle nař. (EU) 2021/1784.</t>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>ZMĚNA sazebního zařazení 8. 9. 2026: z 7616 99 (hliník) → 8536 90 01 00. Zákazník opravil popis: název „magnetic power rail“ byl chybný, nejde o magnetickou hliníkovou lištu, ale o vrchní lištu stojanu s měděnými kontakty (uchycení čistě mechanické). DŮSLEDEK: položka již NENÍ CBAM zboží a odpadá i podezření na antidumping dle nař. (EU) 2021/1784. Opravený popis POTVRZEN KLIENTEM 9. 9. 2026.</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>CBAM zboží (Y137) nebo podmíněný návrh sazebního zařazení – vyžaduje potvrzení před podáním JSD.</t>
+          <t>CBAM zboží – v JSD uvést kód Y137 (výjimka de minimis) u příjemce V-TOP EUROPE s.r.o.</t>
         </is>
       </c>
     </row>
@@ -949,89 +949,101 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Sazebním zařazením z 8. 9. 2026 vyřešeno – dříve chybějící nebo chybný kód.</t>
+          <t>Sazebním zařazením z 8. 9. 2026 změněno nebo doplněno; POTVRZENO KLIENTEM 9. 9. 2026.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>Zdroj HS kódů</t>
+          <t>Stav</t>
         </is>
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>HS_kody_27.8.2026TARIF20260908.xlsx – sazební zařazení ze dne 8. 9. 2026 (sloupec „návrh TC kódu“). Přeškrtnuté kódy v souboru = původní kódy zákazníka, nahrazeny novým návrhem.</t>
+          <t>Celá tabulka POTVRZENA KLIENTEM 9. 9. 2026. Podmíněné návrhy jsou tím uzavřené.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Klasifikace</t>
+          <t>Zdroj HS kódů</t>
         </is>
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Jediný odesílatel (Hangzhou Ontime I.T. Co., Ltd.) → položky sloučeny na unikátní HS kódy. Po přeřazení mají SRCS101, SRCS101D i SR1405 shodný kód 8528 59 00 90 a tvoří jeden řádek.</t>
+          <t>HS_kody_27.8.2026TARIF20260908.xlsx – sazební zařazení ze dne 8. 9. 2026 (sloupec „návrh TC kódu“). Přeškrtnuté kódy v souboru = původní kódy zákazníka, nahrazeny novým návrhem.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>Hrubá hmotnost</t>
+          <t>Klasifikace</t>
         </is>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Sloupec H = hrubá hmotnost kartonů dle packing listu (celkem 714.66 kg). Karton s příslušenstvím (1 CTN, 3,42 kg) obsahuje SRCS101, SRCS101D, SR8100, SR8170 a SR8111 – tára rozpuštěna poměrem k čisté hmotnosti (faktor 1,103226). SR1405 má vlastní karton (1,24 kg).</t>
+          <t>Jediný odesílatel (Hangzhou Ontime I.T. Co., Ltd.) → položky sloučeny na unikátní HS kódy. Po přeřazení mají SRCS101, SRCS101D i SR1405 shodný kód 8528 59 00 90 a tvoří jeden řádek.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>Hrubá hm. vč. palet</t>
+          <t>Hrubá hmotnost</t>
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Sloupec I = sloupec H + poměrný podíl táry 2 palet (30,34 kg), faktor 1.042454. Součet 745.00 kg = deklarovaná hrubá hmotnost dle PL i nákladního listu.</t>
+          <t>Sloupec H = hrubá hmotnost kartonů dle packing listu (celkem 714.66 kg). Karton s příslušenstvím (1 CTN, 3,42 kg) obsahuje SRCS101, SRCS101D, SR8100, SR8170 a SR8111 – tára rozpuštěna poměrem k čisté hmotnosti (faktor 1,103226). SR1405 má vlastní karton (1,24 kg).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>Sleva</t>
+          <t>Hrubá hm. vč. palet</t>
         </is>
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>Faktura PI24200070026046B&amp;051 neobsahuje obchodní slevu (SUB TOTAL = TOTAL = 6 069,20 EUR).</t>
+          <t>Sloupec I = sloupec H + poměrný podíl táry 2 palet (30,34 kg), faktor 1.042454. Součet 745.00 kg = deklarovaná hrubá hmotnost dle PL i nákladního listu.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>Incoterm</t>
+          <t>Sleva</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>CFR Praha (faktura, pole TERMS) – železniční přeprava, FREIGHT PREPAID, CFS-CFS.</t>
+          <t>Faktura PI24200070026046B&amp;051 neobsahuje obchodní slevu (SUB TOTAL = TOTAL = 6 069,20 EUR).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
+          <t>Incoterm</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>CFR Praha (faktura, pole TERMS) – železniční přeprava, FREIGHT PREPAID, CFS-CFS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
           <t>Měna</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>EUR.</t>
         </is>
@@ -1048,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A87"/>
+  <dimension ref="A1:A94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
@@ -1056,560 +1068,604 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="19">
+        <f>== STAV: TABULKA POTVRZENA KLIENTEM 9. 9. 2026 ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>Klient potvrdil sazební zařazení z 8. 9. 2026 v plném rozsahu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tím jsou splněny podmínky u návrhů označených „Pokud popis odpovídá charakteru zboží, pak popisu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>odpovídá navržený TC kód.“ – tj. u SRCS101/SRCS101D, SR1405 a SR8111. Kódy lze použít pro podání JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pozn.: potvrzení klienta se týká správnosti popisu zboží. Nejde o závaznou informaci o sazebním</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>zařazení (ZISZ/BTI) – ta by musela být vydána celním orgánem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="19">
         <f>== ZÁSILKA ===</f>
         <v/>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Odesílatel:   HANGZHOU ONTIME I.T. CO., LTD., 8th Fl, Bldg 6, Realblue Center, #18 Zixuan Rd, Hangzhou 310010, ČÍNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Příjemce (CZ): V-TOP EUROPE s.r.o., Františka Diviše 1012/64, 104 00 Praha 22 – Uhříněves</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>IČO: 257 95 040   |   DIČ / EORI: CZ25795040</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Faktura: PI24200070026046B&amp;051 z 31. 7. 2026   |   P.O. 260021   |   ship date 9. 8. 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Nákladní list (RWB): WPXA26B0812CZ323, Boxline UCL d.o.o., vydáno 12. 8. 2026, Xi'an</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Trasa: Xi'an → Khorgos (ČÍNA) → Praha. Železnice, kontejner CIMU2030715 / 40HC, plomba 328767.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Agent: MAURICE WARD &amp; CO. s.r.o., CTP Logistic Park, Nad Kovárnou 185, 252 68 Kněževes</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Balení: 82 kartonů na 2 paletách   |   GW 745,00 kg   |   NW 665,95 kg   |   3,18 CBM</t>
+          <t>Odesílatel:   HANGZHOU ONTIME I.T. CO., LTD., 8th Fl, Bldg 6, Realblue Center, #18 Zixuan Rd, Hangzhou 310010, ČÍNA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Příjemce (CZ): V-TOP EUROPE s.r.o., Františka Diviše 1012/64, 104 00 Praha 22 – Uhříněves</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IČO: 257 95 040   |   DIČ / EORI: CZ25795040</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Faktura: PI24200070026046B&amp;051 z 31. 7. 2026   |   P.O. 260021   |   ship date 9. 8. 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Nákladní list (RWB): WPXA26B0812CZ323, Boxline UCL d.o.o., vydáno 12. 8. 2026, Xi'an</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Trasa: Xi'an → Khorgos (ČÍNA) → Praha. Železnice, kontejner CIMU2030715 / 40HC, plomba 328767.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agent: MAURICE WARD &amp; CO. s.r.o., CTP Logistic Park, Nad Kovárnou 185, 252 68 Kněževes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Balení: 82 kartonů na 2 paletách   |   GW 745,00 kg   |   NW 665,95 kg   |   3,18 CBM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Hodnota: 6 069,20 EUR   |   Množství: 80 006 ks   |   Incoterm: CFR Praha</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="19">
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19">
         <f>== SAZEBNÍ ZAŘAZENÍ 8. 9. 2026 – ZMĚNY PROTI PŮVODNÍMU SEZNAMU ===</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Zdroj: HS_kody_27.8.2026TARIF20260908.xlsx. V souboru jsou původní kódy přeškrtnuté a nahrazené sloupcem „návrh TC kódu“.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Kód / položka        PŮVODNĚ              NOVĚ                 Změna</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ------------------------------------------------------------------------------------------------------</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  HD2094, HD2051       8531 90 00 00        8531 90 00 00        beze změny (nebylo předmětem posouzení)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SR8100               7616 99              8536 90 01 00        ZMĚNA – CBAM ODPADÁ</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SRCS101, SRCS101D    8531 20 00 00        8528 59 00 90        ZMĚNA</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SR8170               7326 90              7326 90 98 90        doplněno na 10 míst, CBAM trvá</t>
+          <t>Zdroj: HS_kody_27.8.2026TARIF20260908.xlsx. V souboru jsou původní kódy přeškrtnuté a nahrazené sloupcem „návrh TC kódu“.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SR8111               ?                    8504 40 83 90        DOPLNĚNO – chybějící kód vyřešen</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SR1405               8531 20 95 90        8528 59 00 90        ZMĚNA – slučuje se s SRCS101/D</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kód / položka        PŮVODNĚ              NOVĚ                 Změna</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ------------------------------------------------------------------------------------------------------</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t xml:space="preserve">  HD2094, HD2051       8531 90 00 00        8531 90 00 00        beze změny (nebylo předmětem posouzení)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SR8100               7616 99              8536 90 01 00        ZMĚNA – CBAM ODPADÁ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SRCS101, SRCS101D    8531 20 00 00        8528 59 00 90        ZMĚNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SR8170               7326 90              7326 90 98 90        doplněno na 10 míst, CBAM trvá</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SR8111               ?                    8504 40 83 90        DOPLNĚNO – chybějící kód vyřešen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SR1405               8531 20 95 90        8528 59 00 90        ZMĚNA – slučuje se s SRCS101/D</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Počet unikátních HS kódů klesl ze 6 na 5 – SRCS101, SRCS101D a SR1405 mají nyní shodný kód 8528 59 00 90.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="19">
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19">
         <f>== SR8100 – ZÁSADNÍ ZMĚNA, CBAM ODPADÁ ===</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>Zákazník opravil popis produktu: název „magnetic power rail“ byl CHYBNÝ.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Citace ze souboru: „Nakonec se ukázal název produktu SR8100 jako magnetic power rail chybný, nic magnetického</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>v ní není; jedná se o vrchní lištu stojanu pro video tagy, které se do ní uchycují čistě mechanicky</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>(nacvakávají a nasouvají se ze strany), materiál hliník, železo a měď.“</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Nový popis: horizontální napájecí lišta s měděnými kontakty pro mechanické uchycení a napájení LCD video tagů.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>→ Nové zařazení 8536 90 01 00 (elektrická zařízení k spínání/spojování obvodů) místo 7616 99 (výrobky z hliníku).</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>→ DŮSLEDEK 1: položka již NENÍ CBAM zboží (odpadá hliník z přílohy I).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>→ DŮSLEDEK 2: odpadá podezření na antidumpingové clo dle nař. (EU) 2021/1784 (hliníkové profily z ČLR).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="19">
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="19">
         <f>== CBAM – aktualizováno (reference/CBAM_receivers_CZ.xlsx, list List1, řádek 43) ===</f>
         <v/>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>Po přeřazení zůstává v zásilce JEDINÁ CBAM položka:</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • 7326 90 98 90 – stolní kovový stojan SR8170 – čistá hmotnost 1,68 kg (železo/ocel, příloha I)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Dříve uváděná položka 7616 99 (hliník, 0,28 kg) byla přeřazena na 8536 90 01 00 a CBAM se jí již netýká.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Celková čistá hmotnost CBAM zboží v zásilce: 1,68 kg – hluboko pod limitem 50 t/rok.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>PŘÍJEMCE NALEZEN V REGISTRU:</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Firma:                V-TOP EUROPE s.r.o.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   EORI:                 CZ25795040   (shoduje se s DIČ na faktuře)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Y KÓD:                Y137</t>
+          <t xml:space="preserve">   • 7326 90 98 90 – stolní kovový stojan SR8170 – čistá hmotnost 1,68 kg (železo/ocel, příloha I)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Status:               „do 50 t ročně“ – pod limitem de minimis</t>
+          <t>Dříve uváděná položka 7616 99 (hliník, 0,28 kg) byla přeřazena na 8536 90 01 00 a CBAM se jí již netýká.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Povolení (Y128):      není</t>
+          <t>Celková čistá hmotnost CBAM zboží v zásilce: 1,68 kg – hluboko pod limitem 50 t/rok.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Podaná žádost (Y238): není</t>
-        </is>
-      </c>
+      <c r="A48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Datum vydání:         neuvedeno</t>
+          <t>PŘÍJEMCE NALEZEN V REGISTRU:</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Interní reference:    25MWCCCIM008782</t>
+          <t xml:space="preserve">   Firma:                V-TOP EUROPE s.r.o.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>→ Do JSD uvést kód Y137 u položky 7326 90 98 90.</t>
+          <t xml:space="preserve">   EORI:                 CZ25795040   (shoduje se s DIČ na faktuře)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Y KÓD:                Y137</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Status:               „do 50 t ročně“ – pod limitem de minimis</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Povolení (Y128):      není</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Podaná žádost (Y238): není</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Datum vydání:         neuvedeno</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Interní reference:    25MWCCCIM008782</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>→ Do JSD uvést kód Y137 u položky 7326 90 98 90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>→ Příjemce NEPATŘÍ mezi společnosti mimo EU využívající náš sdílený účet CBAM-CZ-2025-QGM67089385721.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="19">
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="19">
         <f>== COO / PREFERENČNÍ VĚTA – TRVÁ ===</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="22" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
         <is>
           <t>!!! V DOKUMENTECH NENÍ ŽÁDNÁ PREFERENČNÍ VĚTA (prohlášení o preferenčním původu). !!!</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Prověřeny: obchodní faktura (2 str.), packing list, železniční nákladní list. Nalezeno pouze „MADE IN CHINA“.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>Země původu: ČÍNA (CN). EU nemá s Čínou dohodu o preferenčním obchodu – preferenční sazba nepřipadá v úvahu.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>→ Uplatní se plné třetizemské (erga omnes) clo u všech položek. Sazby ověřit v TARIC k datu podání JSD.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="19">
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="19">
         <f>== ANTIDUMPING – aktualizováno ===</f>
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="20" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="20" t="inlineStr">
         <is>
           <t>7616 99 – podezření ODPADÁ. Položka byla přeřazena na 8536 90 01 00, nař. (EU) 2021/1784 se neuplatní.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>7326 90 98 90 (stojan SR8170) – u této položky z ČLR není známé antidumpingové opatření; ověřit v TARIC.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>8528 59 00 90, 8504 40 83 90, 8531 90 00 00 – antidumpingová opatření nejsou známa.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="19">
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="19">
         <f>== OTEVŘENÉ BODY PŘED PODÁNÍM JSD ===</f>
         <v/>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="21" t="inlineStr">
-        <is>
-          <t>1) Návrhy u SRCS101/SRCS101D, SR1405 a SR8111 jsou PODMÍNĚNÉ – v souboru je uvedeno:</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   „Pokud popis odpovídá charakteru zboží, pak popisu odpovídá navržený TC kód.“</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   → Nechat klienta potvrdit, že popisy odpovídají skutečnosti, zejména že displeje NEMAJÍ externí</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   obrazový vstup HDMI/DP/VGA/DVI – právě to je důvodem zařazení do 8528 59 místo 8531.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="21" t="inlineStr">
-        <is>
-          <t>2) Přeřazení displejů z položky 8531 do 8528 59 (monitory) může znamenat výrazně vyšší celní sazbu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Dotčená hodnota je 194,00 EUR, dopad tedy malý, ale sazbu je nutné ověřit v TARIC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>3) Kód 8531 90 00 00 (HD etikety, 5 840,00 EUR – 96 % hodnoty zásilky) NEBYL předmětem sazebního</t>
-        </is>
-      </c>
-    </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   zařazení z 8. 9. 2026. Zůstává dle seznamu zákazníka.</t>
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>1) UZAVŘENO – podmíněné návrhy u SRCS101/SRCS101D, SR1405 a SR8111 klient potvrdil 9. 9. 2026,</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>4) Jde o NÁVRH sazebního zařazení, nikoli o závaznou informaci o sazebním zařazení (ZISZ/BTI).</t>
+          <t xml:space="preserve">   včetně toho, že displeje nemají externí obrazový vstup HDMI/DP/VGA/DVI (důvod zařazení do 8528 59).</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
+      <c r="A75" s="21" t="inlineStr">
+        <is>
+          <t>2) Přeřazení displejů z položky 8531 do 8528 59 (monitory) může znamenat výrazně vyšší celní sazbu.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="19">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dotčená hodnota je 194,00 EUR, dopad tedy malý, ale sazbu je nutné ověřit v TARIC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>3) Kód 8531 90 00 00 (HD etikety, 5 840,00 EUR – 96 % hodnoty zásilky) NEBYL předmětem sazebního</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   zařazení z 8. 9. 2026. Zůstává dle seznamu zákazníka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>4) Jde o NÁVRH sazebního zařazení potvrzený klientem, nikoli o závaznou informaci o sazebním</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   zařazení (ZISZ/BTI) vydanou celním orgánem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="22" t="inlineStr">
+        <is>
+          <t>5) TRVÁ: v dokladech chybí preferenční věta – viz sekce COO výše.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="19">
         <f>== HMOTNOSTI – ODVOZENÍ (beze změny) ===</f>
         <v/>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   50 CTN  HD2094                                        GW 365,00   NW 335,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   30 CTN  HD2051                                        GW 345,00   NW 327,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    1 CTN  SRCS101 + SRCS101D + SR8100 + SR8170 + SR8111 GW   3,42   NW   3,10  (sloučená buňka v PL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    1 CTN  SR1405                                        GW   1,24   NW   0,85</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ---------------------------------------------------------------------------------</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   82 CTN                                                GW 714,66   NW 665,95</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   + 2 palety (tára)                                     GW  30,34</t>
-        </is>
-      </c>
-    </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">   = CELKEM                                              GW 745,00   NW 665,95   (3,18 CBM)</t>
+          <t xml:space="preserve">   50 CTN  HD2094                                        GW 365,00   NW 335,00</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Tára kartonu s příslušenstvím rozpuštěna poměrem k čisté hmotnosti (faktor 1,103226),</t>
+          <t xml:space="preserve">   30 CTN  HD2051                                        GW 345,00   NW 327,00</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>tára palet poměrem k hrubé hmotnosti kartonů (faktor 1,042454, sloupec I).</t>
+          <t xml:space="preserve">    1 CTN  SRCS101 + SRCS101D + SR8100 + SR8170 + SR8111 GW   3,42   NW   3,10  (sloučená buňka v PL)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    1 CTN  SR1405                                        GW   1,24   NW   0,85</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ---------------------------------------------------------------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   82 CTN                                                GW 714,66   NW 665,95</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   + 2 palety (tára)                                     GW  30,34</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   = CELKEM                                              GW 745,00   NW 665,95   (3,18 CBM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Tára kartonu s příslušenstvím rozpuštěna poměrem k čisté hmotnosti (faktor 1,103226),</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>tára palet poměrem k hrubé hmotnosti kartonů (faktor 1,042454, sloupec I).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>Kontrola: množství 80 006 ks, čistá hmotnost 665,95 kg i hodnota 6 069,20 EUR souhlasí s doklady.</t>
         </is>

</xml_diff>